<commit_message>
Corrida | SFE-FABO | 2026-06-17 12:03:03.549563
</commit_message>
<xml_diff>
--- a/indicadores/SFE-FABO_out.xlsx
+++ b/indicadores/SFE-FABO_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="538">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Faena de bovinos en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Faena de bovinos</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const | td | easter[8]</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">12/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2124,9 +2130,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2137,7 +2147,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2151,7 +2161,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2167,7 +2177,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2195,7 +2205,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2209,7 +2219,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2237,7 +2247,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2251,7 +2261,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2265,7 +2275,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2279,7 +2289,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2295,7 +2305,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2309,7 +2319,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2457,10 +2467,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2473,10 +2483,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2500,66 +2510,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>35632.7911129417</v>
@@ -2612,7 +2622,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>33770.021648686</v>
@@ -2669,7 +2679,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>39456.3826823136</v>
@@ -2726,7 +2736,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>35191.2081609247</v>
@@ -2783,7 +2793,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>38163.010671338</v>
@@ -2840,7 +2850,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>37711.9685233791</v>
@@ -2897,7 +2907,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>37923.7622276381</v>
@@ -2954,7 +2964,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>39801.9894023353</v>
@@ -3011,7 +3021,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>40543.7287914338</v>
@@ -3068,7 +3078,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>39870.7416069858</v>
@@ -3125,7 +3135,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>42201.3952022187</v>
@@ -3182,7 +3192,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>40884.7212695327</v>
@@ -3239,7 +3249,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>42747.4907337883</v>
@@ -3298,7 +3308,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>40952.0892016063</v>
@@ -3357,7 +3367,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>47650.3534889155</v>
@@ -3416,7 +3426,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>40789.898598018</v>
@@ -3475,7 +3485,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>46577.3115297561</v>
@@ -3534,7 +3544,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>45679.8414757612</v>
@@ -3593,7 +3603,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>44376.0874204592</v>
@@ -3652,7 +3662,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>47855.4565423863</v>
@@ -3711,7 +3721,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>44085.8516035117</v>
@@ -3770,7 +3780,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>41605.9272820745</v>
@@ -3829,7 +3839,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>43617.7367604383</v>
@@ -3888,7 +3898,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>38369.9594215779</v>
@@ -3947,7 +3957,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>45163.2770924978</v>
@@ -4006,7 +4016,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>44296.0303230977</v>
@@ -4065,7 +4075,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>45554.1033833635</v>
@@ -4124,7 +4134,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>43978.3397667093</v>
@@ -4183,7 +4193,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>44673.2446002909</v>
@@ -4242,7 +4252,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>40425.8349103049</v>
@@ -4301,7 +4311,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>45692.7613531452</v>
@@ -4360,7 +4370,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>44584.1897311798</v>
@@ -4419,7 +4429,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>42326.441158328</v>
@@ -4478,7 +4488,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>46633.6052812149</v>
@@ -4537,7 +4547,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>43426.2457206399</v>
@@ -4596,7 +4606,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>41738.5867373565</v>
@@ -4655,7 +4665,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>45669.9694265947</v>
@@ -4714,7 +4724,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>43634.4308227826</v>
@@ -4773,7 +4783,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>45361.9941676137</v>
@@ -4832,7 +4842,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>52279.7363070346</v>
@@ -4891,7 +4901,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>51474.4605728754</v>
@@ -4950,7 +4960,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>47273.2661585694</v>
@@ -5009,7 +5019,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>47696.3811040387</v>
@@ -5068,7 +5078,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>42562.6020339278</v>
@@ -5127,7 +5137,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>44626.2234881029</v>
@@ -5186,7 +5196,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>42827.0488748462</v>
@@ -5245,7 +5255,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>38380.8315911229</v>
@@ -5304,7 +5314,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>39749.1684750605</v>
@@ -5363,7 +5373,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>41045.9397303432</v>
@@ -5422,7 +5432,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>36065.165644018</v>
@@ -5481,7 +5491,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>41267.5998961518</v>
@@ -5540,7 +5550,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>39894.9543737289</v>
@@ -5599,7 +5609,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>38720.4078971919</v>
@@ -5658,7 +5668,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>36590.3773172475</v>
@@ -5717,7 +5727,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>35528.7428463801</v>
@@ -5776,7 +5786,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>36192.6881940569</v>
@@ -5835,7 +5845,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>41521.7411702383</v>
@@ -5894,7 +5904,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>42477.5042967222</v>
@@ -5953,7 +5963,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>43477.6644111632</v>
@@ -6012,7 +6022,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>43287.5221814715</v>
@@ -6071,7 +6081,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>43159.3631053458</v>
@@ -6130,7 +6140,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>38364.9961189575</v>
@@ -6189,7 +6199,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>42779.4217911057</v>
@@ -6248,7 +6258,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>39269.9044891404</v>
@@ -6307,7 +6317,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>41359.3884437053</v>
@@ -6366,7 +6376,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>39562.3810186293</v>
@@ -6425,7 +6435,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>39029.9989379248</v>
@@ -6484,7 +6494,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>40244.1708041182</v>
@@ -6543,7 +6553,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>41943.6522226671</v>
@@ -6602,7 +6612,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>41095.6168586476</v>
@@ -6661,7 +6671,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>44574.1185702851</v>
@@ -6720,7 +6730,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>41896.9170800536</v>
@@ -6779,7 +6789,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>42671.7838719746</v>
@@ -6838,7 +6848,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>39776.0308017078</v>
@@ -6897,7 +6907,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>44393.5622324956</v>
@@ -6956,7 +6966,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>35409.7426833207</v>
@@ -7015,7 +7025,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>40905.2524058624</v>
@@ -7074,7 +7084,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>41088.4098204837</v>
@@ -7133,7 +7143,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>41587.1854143827</v>
@@ -7192,7 +7202,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>38286.6398063509</v>
@@ -7251,7 +7261,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>39520.3334646202</v>
@@ -7310,7 +7320,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>37780.0630834063</v>
@@ -7369,7 +7379,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>39073.5959373033</v>
@@ -7428,7 +7438,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>37021.6066623682</v>
@@ -7487,7 +7497,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>38655.5798962192</v>
@@ -7546,7 +7556,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>36021.958233094</v>
@@ -7605,7 +7615,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>31194.0285348805</v>
@@ -7664,7 +7674,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>28135.7078475315</v>
@@ -7723,7 +7733,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>30456.2012420341</v>
@@ -7782,7 +7792,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>29927.9715465137</v>
@@ -7841,7 +7851,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>31821.6628660675</v>
@@ -7900,7 +7910,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>32869.5523960037</v>
@@ -7959,7 +7969,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>29511.1594715944</v>
@@ -8018,7 +8028,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>33663.3238977391</v>
@@ -8077,7 +8087,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>32512.8636486385</v>
@@ -8136,7 +8146,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>29799.9846958816</v>
@@ -8195,7 +8205,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>29883.0327238997</v>
@@ -8254,7 +8264,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>32668.0983104712</v>
@@ -8313,7 +8323,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>36025.6359190893</v>
@@ -8372,7 +8382,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>37091.3506066536</v>
@@ -8431,7 +8441,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>39809.9689576683</v>
@@ -8490,7 +8500,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>40951.9620115627</v>
@@ -8549,7 +8559,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>41709.0552130838</v>
@@ -8608,7 +8618,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>39392.9611617863</v>
@@ -8667,7 +8677,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>36722.0264822923</v>
@@ -8726,7 +8736,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>37670.7931036793</v>
@@ -8785,7 +8795,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>37646.0954756713</v>
@@ -8844,7 +8854,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>34413.8527321415</v>
@@ -8903,7 +8913,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>38975.9600043358</v>
@@ -8962,7 +8972,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>32879.1775089961</v>
@@ -9021,7 +9031,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>35306.463825984</v>
@@ -9080,7 +9090,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>34396.2375652693</v>
@@ -9139,7 +9149,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>35789.1746651401</v>
@@ -9198,7 +9208,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>38876.7223645644</v>
@@ -9257,7 +9267,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>44125.1782990002</v>
@@ -9316,7 +9326,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>39927.7243865566</v>
@@ -9375,7 +9385,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>43081.6003709658</v>
@@ -9434,7 +9444,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>44931.6071153182</v>
@@ -9493,7 +9503,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>44480.7727230575</v>
@@ -9552,7 +9562,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>44927.3315637011</v>
@@ -9611,7 +9621,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>44395.1946914467</v>
@@ -9670,7 +9680,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>42416.2052037478</v>
@@ -9729,7 +9739,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>48513.8095171329</v>
@@ -9788,7 +9798,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>41171.7672385033</v>
@@ -9847,7 +9857,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>44296.925199289</v>
@@ -9906,7 +9916,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>48614.8249429876</v>
@@ -9965,7 +9975,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>49013.4053450709</v>
@@ -10024,7 +10034,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>47792.8975348261</v>
@@ -10083,7 +10093,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>50050.2697988566</v>
@@ -10142,7 +10152,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>47984.8767543813</v>
@@ -10201,7 +10211,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>49648.2804906289</v>
@@ -10260,7 +10270,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>46782.6847450569</v>
@@ -10319,7 +10329,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>47727.442661591</v>
@@ -10378,7 +10388,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>45162.8690950545</v>
@@ -10437,7 +10447,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>43340.0454751754</v>
@@ -10496,7 +10506,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>46986.9612137702</v>
@@ -10555,7 +10565,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>45631.8355362493</v>
@@ -10614,7 +10624,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>46875.1548299086</v>
@@ -10673,7 +10683,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>46757.8839009054</v>
@@ -10732,7 +10742,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>50813.2911632483</v>
@@ -10791,7 +10801,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>48966.1650683917</v>
@@ -10850,7 +10860,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>47478.2473312182</v>
@@ -10909,7 +10919,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>48436.1670325886</v>
@@ -10968,7 +10978,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>45653.3203579349</v>
@@ -11027,7 +11037,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>45684.1684064876</v>
@@ -11086,7 +11096,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>39678.6499825123</v>
@@ -11145,7 +11155,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>43998.979361883</v>
@@ -11204,7 +11214,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>31613.7815805612</v>
@@ -11263,7 +11273,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>35340.300063398</v>
@@ -11322,7 +11332,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>42234.7542488298</v>
@@ -11381,7 +11391,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>44291.3354166975</v>
@@ -11440,7 +11450,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>49513.8800779989</v>
@@ -11499,7 +11509,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>49459.6222272611</v>
@@ -11558,7 +11568,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>47764.9171173868</v>
@@ -11617,7 +11627,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>48901.0063670352</v>
@@ -11676,7 +11686,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>37204.4271888174</v>
@@ -11735,7 +11745,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>47583.9442</v>
@@ -11794,7 +11804,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>40844.8494</v>
@@ -11853,7 +11863,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>43102.5734</v>
@@ -11912,7 +11922,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>40597.8335</v>
@@ -11971,7 +11981,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>47286.3537</v>
@@ -12030,7 +12040,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>46456.9281</v>
@@ -12089,7 +12099,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>50716.6905</v>
@@ -12148,7 +12158,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>53279.359</v>
@@ -12207,7 +12217,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>41433.5346</v>
@@ -12266,7 +12276,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>49658.0085</v>
@@ -12325,7 +12335,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>55294.6613</v>
@@ -12384,7 +12394,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>45506.364</v>
@@ -12443,7 +12453,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>50241.4763888386</v>
@@ -12502,7 +12512,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>46315.2612445069</v>
@@ -12561,7 +12571,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>26542.9370200079</v>
@@ -12620,7 +12630,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>45986.6923744938</v>
@@ -12679,7 +12689,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>35385.3592367637</v>
@@ -12738,7 +12748,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>33457.7165715508</v>
@@ -12797,7 +12807,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>54450.8464364229</v>
@@ -12856,7 +12866,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>51763.003679407</v>
@@ -12915,7 +12925,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>53195.2088013147</v>
@@ -12974,7 +12984,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>46501.9082129569</v>
@@ -13033,7 +13043,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>43154.1443368487</v>
@@ -13092,7 +13102,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>42095.988447</v>
@@ -13151,7 +13161,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>46809.8162094369</v>
@@ -13210,7 +13220,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>43080.8296027482</v>
@@ -13269,7 +13279,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>44220.4484132247</v>
@@ -13328,7 +13338,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>48944.0597795864</v>
@@ -13387,7 +13397,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>46050.0052600009</v>
@@ -13446,7 +13456,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>52863.5290405046</v>
@@ -13505,7 +13515,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>53651.6840805714</v>
@@ -13564,7 +13574,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>50413.5168465385</v>
@@ -13623,7 +13633,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>46185.9974654813</v>
@@ -13682,7 +13692,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>53364.5308964611</v>
@@ -13741,7 +13751,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>44721.109303197</v>
@@ -13800,7 +13810,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>41496.4161370799</v>
@@ -13859,7 +13869,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>41014.5972711371</v>
@@ -13918,7 +13928,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>37121.9624435967</v>
@@ -13977,7 +13987,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>39961.0598270496</v>
@@ -14036,7 +14046,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>35776.1872</v>
@@ -14095,7 +14105,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>37644.9571813848</v>
@@ -14154,7 +14164,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>36491.4048</v>
@@ -14213,7 +14223,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>38757.2112</v>
@@ -14272,7 +14282,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>42187.296</v>
@@ -14331,7 +14341,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>38471.8968</v>
@@ -14390,7 +14400,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>34539.4778886323</v>
@@ -14449,7 +14459,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>37341.070143816</v>
@@ -14508,7 +14518,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>34500.8251</v>
@@ -14567,7 +14577,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>33392.1473199151</v>
@@ -14626,7 +14636,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>33366.7377195434</v>
@@ -14685,7 +14695,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>36811.7976081183</v>
@@ -14744,7 +14754,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>34727.7677568215</v>
@@ -14803,7 +14813,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>37385.3708153275</v>
@@ -14862,7 +14872,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>35482.436469096</v>
@@ -14921,7 +14931,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>33488.987225017</v>
@@ -14980,7 +14990,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>37643.386159519</v>
@@ -15039,7 +15049,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>39645.823813814</v>
@@ -15098,7 +15108,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>35900.2981596102</v>
@@ -15157,7 +15167,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>34796.1410409335</v>
@@ -15216,7 +15226,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>33522.6440008383</v>
@@ -15275,7 +15285,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>30481.87641178</v>
@@ -15334,7 +15344,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>26370.0753192457</v>
@@ -15393,7 +15403,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>38775.5402931752</v>
@@ -15452,7 +15462,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>35578.2014987737</v>
@@ -15511,7 +15521,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>40369.1884421006</v>
@@ -15570,7 +15580,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>36737.0142891354</v>
@@ -15629,7 +15639,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>38581.0493285534</v>
@@ -15688,7 +15698,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>37901.8971028047</v>
@@ -15747,7 +15757,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>37097.1128256017</v>
@@ -15806,7 +15816,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>39897.191465236</v>
@@ -15865,7 +15875,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>36498.3105051114</v>
@@ -15924,7 +15934,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>34152.1362239935</v>
@@ -15983,7 +15993,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>38334.416132857</v>
@@ -16042,7 +16052,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>33392.7620821494</v>
@@ -16101,7 +16111,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>38958.7848334058</v>
@@ -16160,7 +16170,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>40942.9023182816</v>
@@ -16219,7 +16229,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>42790.039562003</v>
@@ -16278,7 +16288,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>39173.4106918602</v>
@@ -16337,7 +16347,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>44294.5011543204</v>
@@ -16396,7 +16406,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>41901.3619712821</v>
@@ -16455,7 +16465,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>41570.7830001239</v>
@@ -16514,7 +16524,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>40866.5748288959</v>
@@ -16573,7 +16583,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>36432.3692871801</v>
@@ -16632,7 +16642,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>36635.044413362</v>
@@ -16691,7 +16701,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>37398.2212187024</v>
@@ -16750,7 +16760,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>32497.0087971671</v>
@@ -16809,7 +16819,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>37146.1719948126</v>
@@ -16868,7 +16878,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>36281.1473533491</v>
@@ -16927,7 +16937,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>38757.4174362125</v>
@@ -16986,7 +16996,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>39619.5580836204</v>
@@ -17045,7 +17055,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>38302.626689567</v>
@@ -17104,7 +17114,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>36229.4756966555</v>
@@ -17163,7 +17173,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>38945.2625659282</v>
@@ -17222,7 +17232,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>38503.6239452034</v>
@@ -17281,7 +17291,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>33443.0569338259</v>
@@ -17340,7 +17350,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>34800.7581015566</v>
@@ -17399,7 +17409,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>44790.6701404104</v>
@@ -17458,7 +17468,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>39867.979736</v>
@@ -17517,7 +17527,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>44197.3127140851</v>
@@ -17576,7 +17586,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>41658.1451250333</v>
@@ -17635,7 +17645,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>41985.1458304009</v>
@@ -17694,7 +17704,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>47029.8893682832</v>
@@ -17753,7 +17763,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>41816.25774</v>
@@ -17812,7 +17822,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>40413.6514852004</v>
@@ -17871,7 +17881,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>40817.3233894028</v>
@@ -17930,7 +17940,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>39096.1990295</v>
@@ -17989,7 +17999,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>34319.3435854933</v>
@@ -18048,7 +18058,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>33482.1797615297</v>
@@ -18107,7 +18117,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>37611.1337548158</v>
@@ -18166,7 +18176,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>36085.4996191911</v>
@@ -18225,7 +18235,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>40635.4609298501</v>
@@ -18284,7 +18294,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>33478.6942679459</v>
@@ -18343,7 +18353,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>38924.379359928</v>
@@ -18402,7 +18412,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>35429.3202648052</v>
@@ -18461,7 +18471,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>36119.7810608143</v>
@@ -18520,7 +18530,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>41248.8562596469</v>
@@ -18579,7 +18589,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>37986.7465199213</v>
@@ -18638,7 +18648,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>32428.5875275057</v>
@@ -18697,7 +18707,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>37387.4495395079</v>
@@ -18756,7 +18766,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>37299.4705229937</v>
@@ -18815,7 +18825,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>38550.15</v>
@@ -18874,7 +18884,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>33028.744</v>
@@ -18933,7 +18943,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>41045.5125</v>
@@ -18992,7 +19002,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>32951.3625</v>
@@ -19051,7 +19061,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>39792.2155</v>
@@ -19110,7 +19120,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>40928.15675</v>
@@ -19169,7 +19179,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>36214.014</v>
@@ -19228,7 +19238,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>40467.7295</v>
@@ -19287,7 +19297,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>38754.802</v>
@@ -19346,7 +19356,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>41856.895</v>
@@ -19405,7 +19415,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>41437.3745</v>
@@ -19464,7 +19474,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>39139.912</v>
@@ -19523,7 +19533,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>44017.0025</v>
@@ -19582,7 +19592,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>38584.5845</v>
@@ -19641,7 +19651,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>45340.821</v>
@@ -19700,7 +19710,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>42293.979</v>
@@ -19759,7 +19769,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>42966.9505</v>
@@ -19818,7 +19828,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>42116.27475</v>
@@ -19877,7 +19887,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>45356.638</v>
@@ -19936,7 +19946,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>47201.55825</v>
@@ -19995,7 +20005,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>40136.4375</v>
@@ -20054,7 +20064,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>48447.315</v>
@@ -20113,7 +20123,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>44570.922</v>
@@ -20172,7 +20182,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>41424.6</v>
@@ -20231,7 +20241,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>45528.2085</v>
@@ -20290,7 +20300,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>40156.58375</v>
@@ -20349,7 +20359,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>41578.35</v>
@@ -20408,7 +20418,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>43142.918</v>
@@ -20467,7 +20477,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>47603.30825</v>
@@ -20526,7 +20536,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>42526.992</v>
@@ -20585,7 +20595,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>50411.108</v>
@@ -20644,7 +20654,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>48313.8855</v>
@@ -20703,7 +20713,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>50378.766</v>
@@ -20762,7 +20772,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>56333.777</v>
@@ -20821,7 +20831,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>49803.846</v>
@@ -20880,7 +20890,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>49278.117</v>
@@ -20939,7 +20949,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>44959.6125</v>
@@ -20998,7 +21008,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>37433.50475</v>
@@ -21057,7 +21067,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>41632.2045</v>
@@ -21116,7 +21126,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>46695.88</v>
@@ -21175,7 +21185,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>44851.464</v>
@@ -21234,7 +21244,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>47610.855</v>
@@ -21293,7 +21303,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>51059.7865</v>
@@ -21352,7 +21362,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>47632.31</v>
@@ -21411,7 +21421,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>45069.65</v>
@@ -21470,7 +21480,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>48729.699</v>
@@ -21529,7 +21539,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>46832.34</v>
@@ -21588,7 +21598,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>42048.39375</v>
@@ -21647,7 +21657,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>38670.681</v>
@@ -21706,7 +21716,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>37297.4015</v>
@@ -21765,7 +21775,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>46275.647</v>
@@ -21824,7 +21834,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>42997.969</v>
@@ -21883,7 +21893,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>36585.95625</v>
@@ -21942,7 +21952,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>41764.06</v>
@@ -22001,7 +22011,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>44732.5515</v>
@@ -22060,7 +22070,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>45608.4135</v>
@@ -22119,7 +22129,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>44611.63625</v>
@@ -22178,7 +22188,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>42885.78525</v>
@@ -22237,7 +22247,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>42970.095</v>
@@ -22296,7 +22306,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>45189.1425</v>
@@ -22355,7 +22365,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>37138.70475</v>
@@ -22414,7 +22424,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>40857.9475</v>
@@ -22473,7 +22483,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>45267.9185</v>
@@ -22532,7 +22542,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>41404.61325</v>
@@ -22591,7 +22601,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>47160.67</v>
@@ -22650,7 +22660,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>46467.7785</v>
@@ -22709,7 +22719,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>48293.742</v>
@@ -22768,7 +22778,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>50119.202</v>
@@ -22827,7 +22837,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>47930.951</v>
@@ -22886,7 +22896,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>39984.214</v>
@@ -22945,7 +22955,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>44646.994</v>
@@ -23004,7 +23014,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>45809.817</v>
@@ -23063,7 +23073,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>46246.437</v>
@@ -23122,7 +23132,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>39814.60825</v>
@@ -23181,7 +23191,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>49227.27675</v>
@@ -23240,7 +23250,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>43406.832</v>
@@ -23299,7 +23309,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>47693.475</v>
@@ -23358,7 +23368,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>49565.4725</v>
@@ -23417,7 +23427,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>49667.68125</v>
@@ -23476,7 +23486,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>43725.7455</v>
@@ -23535,7 +23545,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>43129.11575</v>
@@ -23594,7 +23604,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>38611.83675</v>
@@ -23653,7 +23663,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>45584.11025</v>
@@ -23712,7 +23722,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>40118.67475</v>
@@ -23771,7 +23781,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>47561.8725</v>
@@ -23830,7 +23840,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>40953.018</v>
@@ -23889,7 +23899,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>41448.9515</v>
@@ -23948,7 +23958,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>38346.4935</v>
@@ -24007,7 +24017,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>44346.039</v>
@@ -24066,7 +24076,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>41183.3585</v>
@@ -24125,7 +24135,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>50240.51</v>
@@ -24184,7 +24194,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>47707.21725</v>
@@ -24243,7 +24253,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>45767.27925</v>
@@ -24302,7 +24312,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>46777.905</v>
@@ -24361,7 +24371,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>42439.635</v>
@@ -24420,7 +24430,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>47279.087</v>
@@ -24479,7 +24489,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>46012.5435</v>
@@ -24538,7 +24548,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>39323.82275</v>
@@ -24597,7 +24607,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>40298.658</v>
@@ -24656,7 +24666,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>43850.80925</v>
@@ -24715,7 +24725,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>47019.614</v>
@@ -24774,7 +24784,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>45424.24425</v>
@@ -24833,7 +24843,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>50325.204</v>
@@ -24892,7 +24902,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>47593.3185</v>
@@ -24951,7 +24961,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>44806.45</v>
@@ -25010,7 +25020,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>45734.276</v>
@@ -25069,7 +25079,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>42549.273</v>
@@ -25128,7 +25138,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>46046.6325</v>
@@ -25187,7 +25197,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>43443.588</v>
@@ -25246,7 +25256,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>38875.122</v>
@@ -25305,7 +25315,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>44642.94</v>
@@ -25364,7 +25374,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>39270.85</v>
@@ -25423,7 +25433,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>43709.04</v>
@@ -25482,7 +25492,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3" t="n">
@@ -25515,7 +25525,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3" t="n">
@@ -25548,7 +25558,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3" t="n">
@@ -25581,7 +25591,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3" t="n">
@@ -25614,7 +25624,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3" t="n">
@@ -25647,7 +25657,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3" t="n">
@@ -25680,7 +25690,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3" t="n">
@@ -25713,7 +25723,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3" t="n">
@@ -25746,7 +25756,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3" t="n">
@@ -25779,7 +25789,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3" t="n">
@@ -25812,7 +25822,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3" t="n">
@@ -25845,7 +25855,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3" t="n">
@@ -25878,7 +25888,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -25901,7 +25911,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -25924,7 +25934,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25947,7 +25957,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25970,7 +25980,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25993,7 +26003,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -26016,7 +26026,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -26039,7 +26049,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -26062,7 +26072,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -26085,7 +26095,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -26108,7 +26118,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -26131,7 +26141,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26154,7 +26164,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26177,7 +26187,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26200,7 +26210,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26223,7 +26233,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26246,7 +26256,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26269,7 +26279,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26292,7 +26302,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26315,7 +26325,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26338,7 +26348,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26361,7 +26371,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26384,7 +26394,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26407,7 +26417,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26430,7 +26440,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26453,7 +26463,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26476,7 +26486,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26499,7 +26509,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26522,7 +26532,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26545,7 +26555,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26568,7 +26578,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -26591,7 +26601,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -26614,7 +26624,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -26637,7 +26647,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -26660,7 +26670,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -26683,7 +26693,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -26706,7 +26716,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -26729,7 +26739,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -26752,7 +26762,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -26775,7 +26785,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -26798,7 +26808,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -26821,7 +26831,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -26844,7 +26854,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -26878,97 +26888,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
   </sheetData>
@@ -26992,7 +27002,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -27002,13 +27012,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.0575913798628941</v>
@@ -27016,7 +27026,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.0338555346052736</v>
@@ -27024,7 +27034,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.0185432629071677</v>
@@ -27032,7 +27042,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>-0.00941459640711278</v>
@@ -27040,7 +27050,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>-0.00588263855079374</v>
@@ -27048,7 +27058,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>-0.0307110870856405</v>
@@ -27056,7 +27066,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>-0.0727235557164664</v>
@@ -27064,7 +27074,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>-0.0543743631197531</v>
@@ -27072,7 +27082,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.0178112252815389</v>
@@ -27080,7 +27090,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.0487457055431213</v>
@@ -27088,7 +27098,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.0131155699099251</v>
@@ -27096,7 +27106,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>-0.0196631719322465</v>
@@ -27104,7 +27114,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>-0.0434569922205234</v>
@@ -27112,7 +27122,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>-0.0591396501992572</v>
@@ -27120,7 +27130,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.0369955399315676</v>
@@ -27128,7 +27138,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.0201198055731067</v>
@@ -27136,7 +27146,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.0306649001491776</v>
@@ -27144,7 +27154,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.0148197134744925</v>
@@ -27152,7 +27162,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.0335284695203665</v>

</xml_diff>